<commit_message>
changes made in files
</commit_message>
<xml_diff>
--- a/data/algonox_data.xlsx
+++ b/data/algonox_data.xlsx
@@ -1460,7 +1460,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:J13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1484,6 +1484,15 @@
       <c r="G1" t="str">
         <v>JoinYear</v>
       </c>
+      <c r="H1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="J1" t="str">
+        <v>LeftYear</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1507,6 +1516,15 @@
       <c r="G2">
         <v>2021</v>
       </c>
+      <c r="H2" t="str">
+        <v>abhishek.kumar@algonox.com</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1530,6 +1548,15 @@
       <c r="G3">
         <v>2022</v>
       </c>
+      <c r="H3" t="str">
+        <v>suresh.babu@algonox.com</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1553,6 +1580,15 @@
       <c r="G4">
         <v>2023</v>
       </c>
+      <c r="H4" t="str">
+        <v>ananya.rao@algonox.com</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1576,6 +1612,15 @@
       <c r="G5">
         <v>2023</v>
       </c>
+      <c r="H5" t="str">
+        <v>kiran.desai@algonox.com</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1599,6 +1644,15 @@
       <c r="G6">
         <v>2020</v>
       </c>
+      <c r="H6" t="str">
+        <v>dileep.varma@algonox.com</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1622,6 +1676,15 @@
       <c r="G7">
         <v>2019</v>
       </c>
+      <c r="H7" t="str">
+        <v>pradeep.nair@algonox.com</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1645,6 +1708,15 @@
       <c r="G8">
         <v>2021</v>
       </c>
+      <c r="H8" t="str">
+        <v>meera.krishnan@algonox.com</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1668,6 +1740,15 @@
       <c r="G9">
         <v>2022</v>
       </c>
+      <c r="H9" t="str">
+        <v>rohan.joshi@algonox.com</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1691,6 +1772,15 @@
       <c r="G10">
         <v>2021</v>
       </c>
+      <c r="H10" t="str">
+        <v>shalini.agarwal@algonox.com</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -1714,10 +1804,83 @@
       <c r="G11">
         <v>2024</v>
       </c>
+      <c r="H11" t="str">
+        <v>mani.bodigam@algonox.com</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>AGX-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Vikram Sinha</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Senior Backend Engineer</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="F12" t="str">
+        <v>ACE Platform, Kafka, Microservices</v>
+      </c>
+      <c r="G12">
+        <v>2020</v>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v>Left</v>
+      </c>
+      <c r="J12">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>AGX-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Pooja Mehta</v>
+      </c>
+      <c r="C13" t="str">
+        <v>AI/ML</v>
+      </c>
+      <c r="D13" t="str">
+        <v>NLP Research Engineer</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Bangalore</v>
+      </c>
+      <c r="F13" t="str">
+        <v>NLP Models, Voice AI, Sweet Hello AI Training</v>
+      </c>
+      <c r="G13">
+        <v>2021</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v>Left</v>
+      </c>
+      <c r="J13">
+        <v>2023</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>